<commit_message>
Add new analysis results and update existing reports
- Added new PNG and PDF files for various analysis results including:
  - INDICADOR_PINZAS_REPARADAS
  - MARCAS_CORRECTIVOS
  - REPORTE_COMPLETO_FASE1
  - REPORTE_MEJORADO_6x2
  - REPUESTOS_CORRECTIVOS_VS_OTROS
  - REPUESTOS_POR_EQUIPO
- Updated README_ANALISIS.md with the new analysis date.
- Updated RESUMEN_CUMPLIMIENTO_FASE1.txt with the new analysis date.
- Added new Excel files for economic summaries and analysis.
- Deleted outdated Excel files related to costs and equipment analysis.
- Updated binary files for various analysis categories and matrices.
</commit_message>
<xml_diff>
--- a/ordenes_filtradas_2025.xlsx
+++ b/ordenes_filtradas_2025.xlsx
@@ -5,16 +5,19 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://udeaeduco-my.sharepoint.com/personal/ana_parra3_udea_edu_co/Documents/UdeA/PROYECTO DE GRADO/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://udeaeduco-my.sharepoint.com/personal/ana_parra3_udea_edu_co/Documents/UdeA/PROYECTO DE GRADO/COPIA 1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{43D63539-3A43-48BB-B421-F136BA3355E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FDFF149D-5BC1-40EE-B477-98160FCA8962}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="8_{43D63539-3A43-48BB-B421-F136BA3355E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A558572C-05E1-47DA-B894-050571315366}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{2B1E2462-8AFB-48CB-AC18-7B6CA8A84C77}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$AJ$414</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -5518,7 +5521,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -5528,6 +5531,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC9C9C9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF79FCD"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -5559,7 +5568,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5569,12 +5578,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="22" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="22" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFF79FCD"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -5883,11 +5902,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86915FE4-2993-48FB-9CAA-1D0CCEED47A1}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:AJ414"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="11" width="11.42578125" style="2"/>
-    <col min="12" max="12" width="102" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="27.7109375" style="2" customWidth="1"/>
     <col min="13" max="20" width="11.42578125" style="2"/>
     <col min="21" max="21" width="18.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="22" max="23" width="11.42578125" style="2"/>
@@ -6008,7 +6028,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>115473</v>
       </c>
@@ -6100,289 +6120,289 @@
       </c>
       <c r="AJ2" s="4"/>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A3" s="3">
+    <row r="3" spans="1:36" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="7">
         <v>117120</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="7">
         <v>1112880233</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="F3" s="4"/>
-      <c r="G3" s="3">
+      <c r="F3" s="8"/>
+      <c r="G3" s="7">
         <v>1000762677</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="I3" s="4"/>
-      <c r="J3" s="3" t="s">
+      <c r="I3" s="8"/>
+      <c r="J3" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="K3" s="4"/>
-      <c r="L3" s="3" t="s">
+      <c r="K3" s="8"/>
+      <c r="L3" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="M3" s="3">
+      <c r="M3" s="7">
         <v>4470</v>
       </c>
-      <c r="N3" s="3">
+      <c r="N3" s="7">
         <v>5954</v>
       </c>
-      <c r="O3" s="4"/>
-      <c r="P3" s="3" t="s">
+      <c r="O3" s="8"/>
+      <c r="P3" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="Q3" s="3" t="s">
+      <c r="Q3" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="R3" s="3" t="s">
+      <c r="R3" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="S3" s="5">
+      <c r="S3" s="9">
         <v>45829</v>
       </c>
-      <c r="T3" s="3" t="s">
+      <c r="T3" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="U3" s="3" t="s">
+      <c r="U3" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="V3" s="4"/>
-      <c r="W3" s="4"/>
-      <c r="X3" s="3" t="s">
+      <c r="V3" s="8"/>
+      <c r="W3" s="8"/>
+      <c r="X3" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="Y3" s="6">
+      <c r="Y3" s="10">
         <v>45828.428807870368</v>
       </c>
-      <c r="Z3" s="4"/>
-      <c r="AA3" s="6">
+      <c r="Z3" s="8"/>
+      <c r="AA3" s="10">
         <v>45828.514398148145</v>
       </c>
-      <c r="AB3" s="6">
+      <c r="AB3" s="10">
         <v>45828.527650462966</v>
       </c>
-      <c r="AC3" s="3">
+      <c r="AC3" s="7">
         <v>19</v>
       </c>
-      <c r="AD3" s="3">
+      <c r="AD3" s="7">
         <v>0</v>
       </c>
-      <c r="AE3" s="3">
+      <c r="AE3" s="7">
         <v>19</v>
       </c>
-      <c r="AF3" s="3">
+      <c r="AF3" s="7">
         <v>255808</v>
       </c>
-      <c r="AG3" s="3" t="s">
+      <c r="AG3" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="AH3" s="6">
+      <c r="AH3" s="10">
         <v>45828.340358796297</v>
       </c>
-      <c r="AI3" s="3" t="s">
+      <c r="AI3" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="AJ3" s="4"/>
+      <c r="AJ3" s="8"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A4" s="3">
+    <row r="4" spans="1:36" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="7">
         <v>123141</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="7">
         <v>1041230037</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="F4" s="4"/>
-      <c r="G4" s="3">
+      <c r="F4" s="8"/>
+      <c r="G4" s="7">
         <v>1000762677</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="I4" s="4"/>
-      <c r="J4" s="3" t="s">
+      <c r="I4" s="8"/>
+      <c r="J4" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="K4" s="4"/>
-      <c r="L4" s="3" t="s">
+      <c r="K4" s="8"/>
+      <c r="L4" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="M4" s="3">
+      <c r="M4" s="7">
         <v>1008</v>
       </c>
-      <c r="N4" s="3">
+      <c r="N4" s="7">
         <v>4175</v>
       </c>
-      <c r="O4" s="4"/>
-      <c r="P4" s="3" t="s">
+      <c r="O4" s="8"/>
+      <c r="P4" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="Q4" s="3" t="s">
+      <c r="Q4" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="R4" s="3" t="s">
+      <c r="R4" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="S4" s="5">
+      <c r="S4" s="9">
         <v>46011</v>
       </c>
-      <c r="T4" s="3" t="s">
+      <c r="T4" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="U4" s="3" t="s">
+      <c r="U4" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="V4" s="4"/>
-      <c r="W4" s="4"/>
-      <c r="X4" s="3" t="s">
+      <c r="V4" s="8"/>
+      <c r="W4" s="8"/>
+      <c r="X4" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="Y4" s="6">
+      <c r="Y4" s="10">
         <v>46008.316874999997</v>
       </c>
-      <c r="Z4" s="4"/>
-      <c r="AA4" s="6">
+      <c r="Z4" s="8"/>
+      <c r="AA4" s="10">
         <v>46008.318298611113</v>
       </c>
-      <c r="AB4" s="6">
+      <c r="AB4" s="10">
         <v>46008.33730324074</v>
       </c>
-      <c r="AC4" s="3">
+      <c r="AC4" s="7">
         <v>27</v>
       </c>
-      <c r="AD4" s="3">
+      <c r="AD4" s="7">
         <v>0</v>
       </c>
-      <c r="AE4" s="3">
+      <c r="AE4" s="7">
         <v>27</v>
       </c>
-      <c r="AF4" s="3">
+      <c r="AF4" s="7">
         <v>266607</v>
       </c>
-      <c r="AG4" s="3" t="s">
+      <c r="AG4" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="AH4" s="6">
+      <c r="AH4" s="10">
         <v>46008.278900462959</v>
       </c>
-      <c r="AI4" s="3" t="s">
+      <c r="AI4" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="AJ4" s="4"/>
+      <c r="AJ4" s="8"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A5" s="3">
+    <row r="5" spans="1:36" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="7">
         <v>118390</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="7">
         <v>1001652414</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="F5" s="4"/>
-      <c r="G5" s="3">
+      <c r="F5" s="8"/>
+      <c r="G5" s="7">
         <v>1000762677</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="H5" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="I5" s="4"/>
-      <c r="J5" s="3" t="s">
+      <c r="I5" s="8"/>
+      <c r="J5" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="K5" s="4"/>
-      <c r="L5" s="3" t="s">
+      <c r="K5" s="8"/>
+      <c r="L5" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="M5" s="3">
+      <c r="M5" s="7">
         <v>986</v>
       </c>
-      <c r="N5" s="3">
+      <c r="N5" s="7">
         <v>3648</v>
       </c>
-      <c r="O5" s="4"/>
-      <c r="P5" s="3" t="s">
+      <c r="O5" s="8"/>
+      <c r="P5" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="Q5" s="3" t="s">
+      <c r="Q5" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="R5" s="3" t="s">
+      <c r="R5" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="S5" s="5">
+      <c r="S5" s="9">
         <v>45871</v>
       </c>
-      <c r="T5" s="3" t="s">
+      <c r="T5" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="U5" s="3" t="s">
+      <c r="U5" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="V5" s="4"/>
-      <c r="W5" s="4"/>
-      <c r="X5" s="3" t="s">
+      <c r="V5" s="8"/>
+      <c r="W5" s="8"/>
+      <c r="X5" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="Y5" s="6">
+      <c r="Y5" s="10">
         <v>45867.603425925925</v>
       </c>
-      <c r="Z5" s="4"/>
-      <c r="AA5" s="6">
+      <c r="Z5" s="8"/>
+      <c r="AA5" s="10">
         <v>45867.64162037037</v>
       </c>
-      <c r="AB5" s="6">
+      <c r="AB5" s="10">
         <v>45867.666805555556</v>
       </c>
-      <c r="AC5" s="3">
+      <c r="AC5" s="7">
         <v>36</v>
       </c>
-      <c r="AD5" s="3">
+      <c r="AD5" s="7">
         <v>0</v>
       </c>
-      <c r="AE5" s="3">
+      <c r="AE5" s="7">
         <v>36</v>
       </c>
-      <c r="AF5" s="3">
+      <c r="AF5" s="7">
         <v>258268</v>
       </c>
-      <c r="AG5" s="3" t="s">
+      <c r="AG5" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="AH5" s="6">
+      <c r="AH5" s="10">
         <v>45867.595243055555</v>
       </c>
-      <c r="AI5" s="3" t="s">
+      <c r="AI5" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="AJ5" s="4"/>
+      <c r="AJ5" s="8"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>113351</v>
       </c>
@@ -6570,7 +6590,7 @@
       </c>
       <c r="AJ7" s="4"/>
     </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>120334</v>
       </c>
@@ -6758,7 +6778,7 @@
       </c>
       <c r="AJ9" s="4"/>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>119500</v>
       </c>
@@ -6854,7 +6874,7 @@
       </c>
       <c r="AJ10" s="4"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>108901</v>
       </c>
@@ -6950,7 +6970,7 @@
       </c>
       <c r="AJ11" s="4"/>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>119059</v>
       </c>
@@ -7046,7 +7066,7 @@
       </c>
       <c r="AJ12" s="4"/>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>113632</v>
       </c>
@@ -7142,7 +7162,7 @@
       </c>
       <c r="AJ13" s="4"/>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>114280</v>
       </c>
@@ -7332,7 +7352,7 @@
       </c>
       <c r="AJ15" s="4"/>
     </row>
-    <row r="16" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>119375</v>
       </c>
@@ -7428,7 +7448,7 @@
       </c>
       <c r="AJ16" s="4"/>
     </row>
-    <row r="17" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>114708</v>
       </c>
@@ -7524,7 +7544,7 @@
       </c>
       <c r="AJ17" s="4"/>
     </row>
-    <row r="18" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>119709</v>
       </c>
@@ -7620,7 +7640,7 @@
       </c>
       <c r="AJ18" s="4"/>
     </row>
-    <row r="19" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>119272</v>
       </c>
@@ -7714,7 +7734,7 @@
       </c>
       <c r="AJ19" s="4"/>
     </row>
-    <row r="20" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>118507</v>
       </c>
@@ -8178,7 +8198,7 @@
       </c>
       <c r="AJ24" s="4"/>
     </row>
-    <row r="25" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>120363</v>
       </c>
@@ -8832,7 +8852,7 @@
       </c>
       <c r="AJ31" s="4"/>
     </row>
-    <row r="32" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3">
         <v>120193</v>
       </c>
@@ -8926,7 +8946,7 @@
       </c>
       <c r="AJ32" s="4"/>
     </row>
-    <row r="33" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
         <v>117433</v>
       </c>
@@ -9020,7 +9040,7 @@
       </c>
       <c r="AJ33" s="4"/>
     </row>
-    <row r="34" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
         <v>123239</v>
       </c>
@@ -9114,7 +9134,7 @@
       </c>
       <c r="AJ34" s="4"/>
     </row>
-    <row r="35" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
         <v>108790</v>
       </c>
@@ -9208,7 +9228,7 @@
       </c>
       <c r="AJ35" s="4"/>
     </row>
-    <row r="36" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>117346</v>
       </c>
@@ -9306,7 +9326,7 @@
       </c>
       <c r="AJ36" s="4"/>
     </row>
-    <row r="37" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>107518</v>
       </c>
@@ -9402,7 +9422,7 @@
       </c>
       <c r="AJ37" s="4"/>
     </row>
-    <row r="38" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="3">
         <v>121000</v>
       </c>
@@ -9500,7 +9520,7 @@
       </c>
       <c r="AJ38" s="4"/>
     </row>
-    <row r="39" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
         <v>119045</v>
       </c>
@@ -9594,7 +9614,7 @@
       </c>
       <c r="AJ39" s="4"/>
     </row>
-    <row r="40" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3">
         <v>118532</v>
       </c>
@@ -9690,7 +9710,7 @@
       </c>
       <c r="AJ40" s="4"/>
     </row>
-    <row r="41" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
         <v>112865</v>
       </c>
@@ -9784,7 +9804,7 @@
       </c>
       <c r="AJ41" s="4"/>
     </row>
-    <row r="42" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="3">
         <v>119254</v>
       </c>
@@ -9878,7 +9898,7 @@
       </c>
       <c r="AJ42" s="4"/>
     </row>
-    <row r="43" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
         <v>123130</v>
       </c>
@@ -9976,7 +9996,7 @@
       </c>
       <c r="AJ43" s="4"/>
     </row>
-    <row r="44" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3">
         <v>123195</v>
       </c>
@@ -10074,7 +10094,7 @@
       </c>
       <c r="AJ44" s="4"/>
     </row>
-    <row r="45" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3">
         <v>121434</v>
       </c>
@@ -10262,7 +10282,7 @@
       </c>
       <c r="AJ46" s="4"/>
     </row>
-    <row r="47" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3">
         <v>120587</v>
       </c>
@@ -10356,7 +10376,7 @@
       </c>
       <c r="AJ47" s="4"/>
     </row>
-    <row r="48" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="3">
         <v>121714</v>
       </c>
@@ -10448,7 +10468,7 @@
       </c>
       <c r="AJ48" s="4"/>
     </row>
-    <row r="49" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3">
         <v>121578</v>
       </c>
@@ -10544,7 +10564,7 @@
       </c>
       <c r="AJ49" s="4"/>
     </row>
-    <row r="50" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="3">
         <v>121624</v>
       </c>
@@ -10638,7 +10658,7 @@
       </c>
       <c r="AJ50" s="4"/>
     </row>
-    <row r="51" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="3">
         <v>124880</v>
       </c>
@@ -10732,7 +10752,7 @@
       </c>
       <c r="AJ51" s="4"/>
     </row>
-    <row r="52" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="3">
         <v>121848</v>
       </c>
@@ -10820,7 +10840,7 @@
       </c>
       <c r="AJ52" s="4"/>
     </row>
-    <row r="53" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="3">
         <v>116723</v>
       </c>
@@ -10916,7 +10936,7 @@
       </c>
       <c r="AJ53" s="4"/>
     </row>
-    <row r="54" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="3">
         <v>113737</v>
       </c>
@@ -11010,7 +11030,7 @@
       </c>
       <c r="AJ54" s="4"/>
     </row>
-    <row r="55" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="3">
         <v>108496</v>
       </c>
@@ -11104,7 +11124,7 @@
       </c>
       <c r="AJ55" s="4"/>
     </row>
-    <row r="56" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3">
         <v>113604</v>
       </c>
@@ -11292,7 +11312,7 @@
       </c>
       <c r="AJ57" s="4"/>
     </row>
-    <row r="58" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="3">
         <v>115096</v>
       </c>
@@ -11386,7 +11406,7 @@
       </c>
       <c r="AJ58" s="4"/>
     </row>
-    <row r="59" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="3">
         <v>116296</v>
       </c>
@@ -11482,7 +11502,7 @@
       </c>
       <c r="AJ59" s="4"/>
     </row>
-    <row r="60" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="3">
         <v>113729</v>
       </c>
@@ -11672,7 +11692,7 @@
       </c>
       <c r="AJ61" s="4"/>
     </row>
-    <row r="62" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="3">
         <v>118666</v>
       </c>
@@ -11860,7 +11880,7 @@
       </c>
       <c r="AJ63" s="4"/>
     </row>
-    <row r="64" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="3">
         <v>115823</v>
       </c>
@@ -11954,7 +11974,7 @@
       </c>
       <c r="AJ64" s="4"/>
     </row>
-    <row r="65" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3">
         <v>113548</v>
       </c>
@@ -12050,7 +12070,7 @@
       </c>
       <c r="AJ65" s="4"/>
     </row>
-    <row r="66" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="3">
         <v>113673</v>
       </c>
@@ -12148,7 +12168,7 @@
       </c>
       <c r="AJ66" s="4"/>
     </row>
-    <row r="67" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="3">
         <v>116386</v>
       </c>
@@ -12244,7 +12264,7 @@
       </c>
       <c r="AJ67" s="4"/>
     </row>
-    <row r="68" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="3">
         <v>109188</v>
       </c>
@@ -12340,7 +12360,7 @@
       </c>
       <c r="AJ68" s="4"/>
     </row>
-    <row r="69" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="3">
         <v>117684</v>
       </c>
@@ -12434,7 +12454,7 @@
       </c>
       <c r="AJ69" s="4"/>
     </row>
-    <row r="70" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="3">
         <v>117793</v>
       </c>
@@ -12526,7 +12546,7 @@
       </c>
       <c r="AJ70" s="4"/>
     </row>
-    <row r="71" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="3">
         <v>116917</v>
       </c>
@@ -12716,7 +12736,7 @@
       </c>
       <c r="AJ72" s="4"/>
     </row>
-    <row r="73" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="3">
         <v>116140</v>
       </c>
@@ -12810,7 +12830,7 @@
       </c>
       <c r="AJ73" s="4"/>
     </row>
-    <row r="74" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="3">
         <v>116838</v>
       </c>
@@ -12906,7 +12926,7 @@
       </c>
       <c r="AJ74" s="4"/>
     </row>
-    <row r="75" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="3">
         <v>116797</v>
       </c>
@@ -13090,7 +13110,7 @@
       </c>
       <c r="AJ76" s="4"/>
     </row>
-    <row r="77" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="3">
         <v>116391</v>
       </c>
@@ -13182,7 +13202,7 @@
       </c>
       <c r="AJ77" s="4"/>
     </row>
-    <row r="78" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="3">
         <v>118766</v>
       </c>
@@ -13276,7 +13296,7 @@
       </c>
       <c r="AJ78" s="4"/>
     </row>
-    <row r="79" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="3">
         <v>108060</v>
       </c>
@@ -13372,7 +13392,7 @@
       </c>
       <c r="AJ79" s="4"/>
     </row>
-    <row r="80" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="3">
         <v>117754</v>
       </c>
@@ -13466,7 +13486,7 @@
       </c>
       <c r="AJ80" s="4"/>
     </row>
-    <row r="81" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="3">
         <v>113458</v>
       </c>
@@ -13654,7 +13674,7 @@
       </c>
       <c r="AJ82" s="4"/>
     </row>
-    <row r="83" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="3">
         <v>118767</v>
       </c>
@@ -13748,7 +13768,7 @@
       </c>
       <c r="AJ83" s="4"/>
     </row>
-    <row r="84" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="3">
         <v>116881</v>
       </c>
@@ -13844,7 +13864,7 @@
       </c>
       <c r="AJ84" s="4"/>
     </row>
-    <row r="85" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="3">
         <v>116468</v>
       </c>
@@ -13936,7 +13956,7 @@
       </c>
       <c r="AJ85" s="4"/>
     </row>
-    <row r="86" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" s="3">
         <v>115871</v>
       </c>
@@ -14032,7 +14052,7 @@
       </c>
       <c r="AJ86" s="4"/>
     </row>
-    <row r="87" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="3">
         <v>115844</v>
       </c>
@@ -14128,7 +14148,7 @@
       </c>
       <c r="AJ87" s="4"/>
     </row>
-    <row r="88" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" s="3">
         <v>111237</v>
       </c>
@@ -14224,7 +14244,7 @@
       </c>
       <c r="AJ88" s="4"/>
     </row>
-    <row r="89" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="3">
         <v>108520</v>
       </c>
@@ -14414,7 +14434,7 @@
       </c>
       <c r="AJ90" s="4"/>
     </row>
-    <row r="91" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="3">
         <v>114927</v>
       </c>
@@ -14508,7 +14528,7 @@
       </c>
       <c r="AJ91" s="4"/>
     </row>
-    <row r="92" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="3">
         <v>117832</v>
       </c>
@@ -14882,7 +14902,7 @@
       </c>
       <c r="AJ95" s="4"/>
     </row>
-    <row r="96" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" s="3">
         <v>114706</v>
       </c>
@@ -14976,7 +14996,7 @@
       </c>
       <c r="AJ96" s="4"/>
     </row>
-    <row r="97" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" s="3">
         <v>118665</v>
       </c>
@@ -15070,7 +15090,7 @@
       </c>
       <c r="AJ97" s="4"/>
     </row>
-    <row r="98" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" s="3">
         <v>114495</v>
       </c>
@@ -15164,7 +15184,7 @@
       </c>
       <c r="AJ98" s="4"/>
     </row>
-    <row r="99" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" s="3">
         <v>106640</v>
       </c>
@@ -15254,7 +15274,7 @@
       </c>
       <c r="AJ99" s="4"/>
     </row>
-    <row r="100" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" s="3">
         <v>118312</v>
       </c>
@@ -15350,7 +15370,7 @@
       </c>
       <c r="AJ100" s="4"/>
     </row>
-    <row r="101" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" s="3">
         <v>115117</v>
       </c>
@@ -15444,7 +15464,7 @@
       </c>
       <c r="AJ101" s="4"/>
     </row>
-    <row r="102" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" s="3">
         <v>116879</v>
       </c>
@@ -15538,7 +15558,7 @@
       </c>
       <c r="AJ102" s="4"/>
     </row>
-    <row r="103" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3">
         <v>115793</v>
       </c>
@@ -15632,7 +15652,7 @@
       </c>
       <c r="AJ103" s="4"/>
     </row>
-    <row r="104" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" s="3">
         <v>121155</v>
       </c>
@@ -15720,7 +15740,7 @@
       </c>
       <c r="AJ104" s="4"/>
     </row>
-    <row r="105" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" s="3">
         <v>121952</v>
       </c>
@@ -15810,7 +15830,7 @@
       </c>
       <c r="AJ105" s="4"/>
     </row>
-    <row r="106" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106" s="3">
         <v>112641</v>
       </c>
@@ -15906,7 +15926,7 @@
       </c>
       <c r="AJ106" s="4"/>
     </row>
-    <row r="107" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107" s="3">
         <v>114406</v>
       </c>
@@ -16096,7 +16116,7 @@
       </c>
       <c r="AJ108" s="4"/>
     </row>
-    <row r="109" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" s="3">
         <v>108379</v>
       </c>
@@ -16190,7 +16210,7 @@
       </c>
       <c r="AJ109" s="4"/>
     </row>
-    <row r="110" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" s="3">
         <v>108397</v>
       </c>
@@ -16286,7 +16306,7 @@
       </c>
       <c r="AJ110" s="4"/>
     </row>
-    <row r="111" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" s="3">
         <v>106698</v>
       </c>
@@ -16382,7 +16402,7 @@
       </c>
       <c r="AJ111" s="4"/>
     </row>
-    <row r="112" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112" s="3">
         <v>107619</v>
       </c>
@@ -16478,7 +16498,7 @@
       </c>
       <c r="AJ112" s="4"/>
     </row>
-    <row r="113" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" s="3">
         <v>107263</v>
       </c>
@@ -16668,7 +16688,7 @@
       </c>
       <c r="AJ114" s="4"/>
     </row>
-    <row r="115" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115" s="3">
         <v>107186</v>
       </c>
@@ -16858,7 +16878,7 @@
       </c>
       <c r="AJ116" s="4"/>
     </row>
-    <row r="117" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" s="3">
         <v>111308</v>
       </c>
@@ -16952,7 +16972,7 @@
       </c>
       <c r="AJ117" s="4"/>
     </row>
-    <row r="118" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" s="3">
         <v>107923</v>
       </c>
@@ -17050,7 +17070,7 @@
       </c>
       <c r="AJ118" s="4"/>
     </row>
-    <row r="119" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" s="3">
         <v>111636</v>
       </c>
@@ -17144,7 +17164,7 @@
       </c>
       <c r="AJ119" s="4"/>
     </row>
-    <row r="120" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120" s="3">
         <v>112808</v>
       </c>
@@ -17238,7 +17258,7 @@
       </c>
       <c r="AJ120" s="4"/>
     </row>
-    <row r="121" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121" s="3">
         <v>114231</v>
       </c>
@@ -17426,7 +17446,7 @@
       </c>
       <c r="AJ122" s="4"/>
     </row>
-    <row r="123" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123" s="3">
         <v>106687</v>
       </c>
@@ -17710,7 +17730,7 @@
       </c>
       <c r="AJ125" s="4"/>
     </row>
-    <row r="126" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126" s="3">
         <v>107199</v>
       </c>
@@ -17900,7 +17920,7 @@
       </c>
       <c r="AJ127" s="4"/>
     </row>
-    <row r="128" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A128" s="3">
         <v>112102</v>
       </c>
@@ -18090,7 +18110,7 @@
       </c>
       <c r="AJ129" s="4"/>
     </row>
-    <row r="130" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A130" s="3">
         <v>111307</v>
       </c>
@@ -18184,7 +18204,7 @@
       </c>
       <c r="AJ130" s="4"/>
     </row>
-    <row r="131" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131" s="3">
         <v>111238</v>
       </c>
@@ -18466,7 +18486,7 @@
       </c>
       <c r="AJ133" s="4"/>
     </row>
-    <row r="134" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A134" s="3">
         <v>112810</v>
       </c>
@@ -18562,7 +18582,7 @@
       </c>
       <c r="AJ134" s="4"/>
     </row>
-    <row r="135" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A135" s="3">
         <v>107204</v>
       </c>
@@ -18656,7 +18676,7 @@
       </c>
       <c r="AJ135" s="4"/>
     </row>
-    <row r="136" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A136" s="3">
         <v>114087</v>
       </c>
@@ -18752,7 +18772,7 @@
       </c>
       <c r="AJ136" s="4"/>
     </row>
-    <row r="137" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137" s="3">
         <v>107188</v>
       </c>
@@ -18940,7 +18960,7 @@
       </c>
       <c r="AJ138" s="4"/>
     </row>
-    <row r="139" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139" s="3">
         <v>107704</v>
       </c>
@@ -19604,7 +19624,7 @@
       </c>
       <c r="AJ145" s="4"/>
     </row>
-    <row r="146" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A146" s="3">
         <v>112680</v>
       </c>
@@ -19698,7 +19718,7 @@
       </c>
       <c r="AJ146" s="4"/>
     </row>
-    <row r="147" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A147" s="3">
         <v>112200</v>
       </c>
@@ -19792,7 +19812,7 @@
       </c>
       <c r="AJ147" s="4"/>
     </row>
-    <row r="148" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A148" s="3">
         <v>111241</v>
       </c>
@@ -19978,7 +19998,7 @@
       </c>
       <c r="AJ149" s="4"/>
     </row>
-    <row r="150" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150" s="3">
         <v>106679</v>
       </c>
@@ -20072,7 +20092,7 @@
       </c>
       <c r="AJ150" s="4"/>
     </row>
-    <row r="151" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A151" s="3">
         <v>112766</v>
       </c>
@@ -20358,7 +20378,7 @@
       </c>
       <c r="AJ153" s="4"/>
     </row>
-    <row r="154" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154" s="3">
         <v>121543</v>
       </c>
@@ -20452,7 +20472,7 @@
       </c>
       <c r="AJ154" s="4"/>
     </row>
-    <row r="155" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A155" s="3">
         <v>121052</v>
       </c>
@@ -20642,7 +20662,7 @@
       </c>
       <c r="AJ156" s="4"/>
     </row>
-    <row r="157" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157" s="3">
         <v>121088</v>
       </c>
@@ -20738,7 +20758,7 @@
       </c>
       <c r="AJ157" s="4"/>
     </row>
-    <row r="158" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A158" s="3">
         <v>121297</v>
       </c>
@@ -20928,7 +20948,7 @@
       </c>
       <c r="AJ159" s="4"/>
     </row>
-    <row r="160" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A160" s="3">
         <v>121161</v>
       </c>
@@ -21116,7 +21136,7 @@
       </c>
       <c r="AJ161" s="4"/>
     </row>
-    <row r="162" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A162" s="3">
         <v>121774</v>
       </c>
@@ -21304,7 +21324,7 @@
       </c>
       <c r="AJ163" s="4"/>
     </row>
-    <row r="164" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A164" s="3">
         <v>121726</v>
       </c>
@@ -21396,7 +21416,7 @@
       </c>
       <c r="AJ164" s="4"/>
     </row>
-    <row r="165" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A165" s="3">
         <v>121668</v>
       </c>
@@ -21492,7 +21512,7 @@
       </c>
       <c r="AJ165" s="4"/>
     </row>
-    <row r="166" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A166" s="3">
         <v>121949</v>
       </c>
@@ -21586,7 +21606,7 @@
       </c>
       <c r="AJ166" s="4"/>
     </row>
-    <row r="167" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A167" s="3">
         <v>121087</v>
       </c>
@@ -21682,7 +21702,7 @@
       </c>
       <c r="AJ167" s="4"/>
     </row>
-    <row r="168" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A168" s="3">
         <v>121163</v>
       </c>
@@ -21774,7 +21794,7 @@
       </c>
       <c r="AJ168" s="4"/>
     </row>
-    <row r="169" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A169" s="3">
         <v>120959</v>
       </c>
@@ -21870,7 +21890,7 @@
       </c>
       <c r="AJ169" s="4"/>
     </row>
-    <row r="170" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A170" s="3">
         <v>115327</v>
       </c>
@@ -21966,7 +21986,7 @@
       </c>
       <c r="AJ170" s="4"/>
     </row>
-    <row r="171" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A171" s="3">
         <v>114099</v>
       </c>
@@ -22064,7 +22084,7 @@
       </c>
       <c r="AJ171" s="4"/>
     </row>
-    <row r="172" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A172" s="3">
         <v>117421</v>
       </c>
@@ -22160,7 +22180,7 @@
       </c>
       <c r="AJ172" s="4"/>
     </row>
-    <row r="173" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A173" s="3">
         <v>121090</v>
       </c>
@@ -22258,7 +22278,7 @@
       </c>
       <c r="AJ173" s="4"/>
     </row>
-    <row r="174" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A174" s="3">
         <v>120316</v>
       </c>
@@ -22358,7 +22378,7 @@
       </c>
       <c r="AJ174" s="4"/>
     </row>
-    <row r="175" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A175" s="3">
         <v>111427</v>
       </c>
@@ -22448,7 +22468,7 @@
       </c>
       <c r="AJ175" s="4"/>
     </row>
-    <row r="176" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A176" s="3">
         <v>113925</v>
       </c>
@@ -22538,7 +22558,7 @@
       </c>
       <c r="AJ176" s="4"/>
     </row>
-    <row r="177" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A177" s="3">
         <v>114768</v>
       </c>
@@ -22626,7 +22646,7 @@
       </c>
       <c r="AJ177" s="4"/>
     </row>
-    <row r="178" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A178" s="3">
         <v>106645</v>
       </c>
@@ -22724,7 +22744,7 @@
       </c>
       <c r="AJ178" s="4"/>
     </row>
-    <row r="179" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A179" s="3">
         <v>107519</v>
       </c>
@@ -22820,7 +22840,7 @@
       </c>
       <c r="AJ179" s="4"/>
     </row>
-    <row r="180" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A180" s="3">
         <v>117906</v>
       </c>
@@ -22916,7 +22936,7 @@
       </c>
       <c r="AJ180" s="4"/>
     </row>
-    <row r="181" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A181" s="3">
         <v>120225</v>
       </c>
@@ -23010,7 +23030,7 @@
       </c>
       <c r="AJ181" s="4"/>
     </row>
-    <row r="182" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A182" s="3">
         <v>118144</v>
       </c>
@@ -23104,7 +23124,7 @@
       </c>
       <c r="AJ182" s="4"/>
     </row>
-    <row r="183" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A183" s="3">
         <v>121157</v>
       </c>
@@ -23388,7 +23408,7 @@
       </c>
       <c r="AJ185" s="4"/>
     </row>
-    <row r="186" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A186" s="3">
         <v>120540</v>
       </c>
@@ -23576,7 +23596,7 @@
       </c>
       <c r="AJ187" s="4"/>
     </row>
-    <row r="188" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A188" s="3">
         <v>119464</v>
       </c>
@@ -23952,7 +23972,7 @@
       </c>
       <c r="AJ191" s="4"/>
     </row>
-    <row r="192" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A192" s="3">
         <v>120085</v>
       </c>
@@ -24422,7 +24442,7 @@
       </c>
       <c r="AJ196" s="4"/>
     </row>
-    <row r="197" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A197" s="3">
         <v>120206</v>
       </c>
@@ -24516,7 +24536,7 @@
       </c>
       <c r="AJ197" s="4"/>
     </row>
-    <row r="198" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A198" s="3">
         <v>120228</v>
       </c>
@@ -24610,7 +24630,7 @@
       </c>
       <c r="AJ198" s="4"/>
     </row>
-    <row r="199" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A199" s="3">
         <v>119267</v>
       </c>
@@ -24702,7 +24722,7 @@
       </c>
       <c r="AJ199" s="4"/>
     </row>
-    <row r="200" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A200" s="3">
         <v>118145</v>
       </c>
@@ -24796,7 +24816,7 @@
       </c>
       <c r="AJ200" s="4"/>
     </row>
-    <row r="201" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A201" s="3">
         <v>118178</v>
       </c>
@@ -24986,7 +25006,7 @@
       </c>
       <c r="AJ202" s="4"/>
     </row>
-    <row r="203" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A203" s="3">
         <v>119418</v>
       </c>
@@ -25174,7 +25194,7 @@
       </c>
       <c r="AJ204" s="4"/>
     </row>
-    <row r="205" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A205" s="3">
         <v>120795</v>
       </c>
@@ -25268,7 +25288,7 @@
       </c>
       <c r="AJ205" s="4"/>
     </row>
-    <row r="206" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A206" s="3">
         <v>121066</v>
       </c>
@@ -25366,7 +25386,7 @@
       </c>
       <c r="AJ206" s="4"/>
     </row>
-    <row r="207" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A207" s="3">
         <v>120788</v>
       </c>
@@ -25460,7 +25480,7 @@
       </c>
       <c r="AJ207" s="4"/>
     </row>
-    <row r="208" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A208" s="3">
         <v>118282</v>
       </c>
@@ -25552,7 +25572,7 @@
       </c>
       <c r="AJ208" s="4"/>
     </row>
-    <row r="209" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A209" s="3">
         <v>121150</v>
       </c>
@@ -25834,7 +25854,7 @@
       </c>
       <c r="AJ211" s="4"/>
     </row>
-    <row r="212" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A212" s="3">
         <v>117692</v>
       </c>
@@ -26024,7 +26044,7 @@
       </c>
       <c r="AJ213" s="4"/>
     </row>
-    <row r="214" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A214" s="3">
         <v>118433</v>
       </c>
@@ -26212,7 +26232,7 @@
       </c>
       <c r="AJ215" s="4"/>
     </row>
-    <row r="216" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A216" s="3">
         <v>118353</v>
       </c>
@@ -26306,7 +26326,7 @@
       </c>
       <c r="AJ216" s="4"/>
     </row>
-    <row r="217" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A217" s="3">
         <v>116986</v>
       </c>
@@ -26400,7 +26420,7 @@
       </c>
       <c r="AJ217" s="4"/>
     </row>
-    <row r="218" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A218" s="3">
         <v>118863</v>
       </c>
@@ -26684,7 +26704,7 @@
       </c>
       <c r="AJ220" s="4"/>
     </row>
-    <row r="221" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A221" s="3">
         <v>119030</v>
       </c>
@@ -27060,7 +27080,7 @@
       </c>
       <c r="AJ224" s="4"/>
     </row>
-    <row r="225" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A225" s="3">
         <v>118619</v>
       </c>
@@ -27156,7 +27176,7 @@
       </c>
       <c r="AJ225" s="4"/>
     </row>
-    <row r="226" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A226" s="3">
         <v>118489</v>
       </c>
@@ -27250,7 +27270,7 @@
       </c>
       <c r="AJ226" s="4"/>
     </row>
-    <row r="227" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A227" s="3">
         <v>117689</v>
       </c>
@@ -27344,7 +27364,7 @@
       </c>
       <c r="AJ227" s="4"/>
     </row>
-    <row r="228" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A228" s="3">
         <v>118462</v>
       </c>
@@ -27438,7 +27458,7 @@
       </c>
       <c r="AJ228" s="4"/>
     </row>
-    <row r="229" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A229" s="3">
         <v>118658</v>
       </c>
@@ -27532,7 +27552,7 @@
       </c>
       <c r="AJ229" s="4"/>
     </row>
-    <row r="230" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A230" s="3">
         <v>108384</v>
       </c>
@@ -27626,7 +27646,7 @@
       </c>
       <c r="AJ230" s="4"/>
     </row>
-    <row r="231" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A231" s="3">
         <v>115752</v>
       </c>
@@ -27724,7 +27744,7 @@
       </c>
       <c r="AJ231" s="4"/>
     </row>
-    <row r="232" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A232" s="3">
         <v>114024</v>
       </c>
@@ -27818,7 +27838,7 @@
       </c>
       <c r="AJ232" s="4"/>
     </row>
-    <row r="233" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A233" s="3">
         <v>120669</v>
       </c>
@@ -27914,7 +27934,7 @@
       </c>
       <c r="AJ233" s="4"/>
     </row>
-    <row r="234" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A234" s="3">
         <v>120472</v>
       </c>
@@ -28008,7 +28028,7 @@
       </c>
       <c r="AJ234" s="4"/>
     </row>
-    <row r="235" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A235" s="3">
         <v>114017</v>
       </c>
@@ -28102,7 +28122,7 @@
       </c>
       <c r="AJ235" s="4"/>
     </row>
-    <row r="236" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A236" s="3">
         <v>119511</v>
       </c>
@@ -28292,7 +28312,7 @@
       </c>
       <c r="AJ237" s="4"/>
     </row>
-    <row r="238" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A238" s="3">
         <v>117069</v>
       </c>
@@ -28386,7 +28406,7 @@
       </c>
       <c r="AJ238" s="4"/>
     </row>
-    <row r="239" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A239" s="3">
         <v>123205</v>
       </c>
@@ -28480,7 +28500,7 @@
       </c>
       <c r="AJ239" s="4"/>
     </row>
-    <row r="240" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A240" s="3">
         <v>108382</v>
       </c>
@@ -28574,7 +28594,7 @@
       </c>
       <c r="AJ240" s="4"/>
     </row>
-    <row r="241" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A241" s="3">
         <v>121466</v>
       </c>
@@ -28668,7 +28688,7 @@
       </c>
       <c r="AJ241" s="4"/>
     </row>
-    <row r="242" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A242" s="3">
         <v>121604</v>
       </c>
@@ -28762,7 +28782,7 @@
       </c>
       <c r="AJ242" s="4"/>
     </row>
-    <row r="243" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A243" s="3">
         <v>119650</v>
       </c>
@@ -28856,7 +28876,7 @@
       </c>
       <c r="AJ243" s="4"/>
     </row>
-    <row r="244" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A244" s="3">
         <v>119514</v>
       </c>
@@ -28952,7 +28972,7 @@
       </c>
       <c r="AJ244" s="4"/>
     </row>
-    <row r="245" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A245" s="3">
         <v>108504</v>
       </c>
@@ -29048,7 +29068,7 @@
       </c>
       <c r="AJ245" s="4"/>
     </row>
-    <row r="246" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A246" s="3">
         <v>115945</v>
       </c>
@@ -29142,7 +29162,7 @@
       </c>
       <c r="AJ246" s="4"/>
     </row>
-    <row r="247" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A247" s="3">
         <v>116945</v>
       </c>
@@ -29236,7 +29256,7 @@
       </c>
       <c r="AJ247" s="4"/>
     </row>
-    <row r="248" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A248" s="3">
         <v>119513</v>
       </c>
@@ -29332,7 +29352,7 @@
       </c>
       <c r="AJ248" s="4"/>
     </row>
-    <row r="249" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A249" s="3">
         <v>117080</v>
       </c>
@@ -29616,7 +29636,7 @@
       </c>
       <c r="AJ251" s="4"/>
     </row>
-    <row r="252" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A252" s="3">
         <v>117039</v>
       </c>
@@ -30468,7 +30488,7 @@
       </c>
       <c r="AJ260" s="4"/>
     </row>
-    <row r="261" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A261" s="3">
         <v>120023</v>
       </c>
@@ -30564,7 +30584,7 @@
       </c>
       <c r="AJ261" s="4"/>
     </row>
-    <row r="262" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A262" s="3">
         <v>117493</v>
       </c>
@@ -30658,7 +30678,7 @@
       </c>
       <c r="AJ262" s="4"/>
     </row>
-    <row r="263" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A263" s="3">
         <v>118541</v>
       </c>
@@ -30752,7 +30772,7 @@
       </c>
       <c r="AJ263" s="4"/>
     </row>
-    <row r="264" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A264" s="3">
         <v>112827</v>
       </c>
@@ -30846,7 +30866,7 @@
       </c>
       <c r="AJ264" s="4"/>
     </row>
-    <row r="265" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A265" s="3">
         <v>121212</v>
       </c>
@@ -30940,7 +30960,7 @@
       </c>
       <c r="AJ265" s="4"/>
     </row>
-    <row r="266" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A266" s="3">
         <v>123396</v>
       </c>
@@ -31032,7 +31052,7 @@
       </c>
       <c r="AJ266" s="4"/>
     </row>
-    <row r="267" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A267" s="3">
         <v>108231</v>
       </c>
@@ -31222,7 +31242,7 @@
       </c>
       <c r="AJ268" s="4"/>
     </row>
-    <row r="269" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A269" s="3">
         <v>117298</v>
       </c>
@@ -31318,7 +31338,7 @@
       </c>
       <c r="AJ269" s="4"/>
     </row>
-    <row r="270" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A270" s="3">
         <v>119938</v>
       </c>
@@ -31412,7 +31432,7 @@
       </c>
       <c r="AJ270" s="4"/>
     </row>
-    <row r="271" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A271" s="3">
         <v>108385</v>
       </c>
@@ -31506,7 +31526,7 @@
       </c>
       <c r="AJ271" s="4"/>
     </row>
-    <row r="272" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A272" s="3">
         <v>117550</v>
       </c>
@@ -31600,7 +31620,7 @@
       </c>
       <c r="AJ272" s="4"/>
     </row>
-    <row r="273" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A273" s="3">
         <v>119603</v>
       </c>
@@ -31788,7 +31808,7 @@
       </c>
       <c r="AJ274" s="4"/>
     </row>
-    <row r="275" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A275" s="3">
         <v>113336</v>
       </c>
@@ -31978,7 +31998,7 @@
       </c>
       <c r="AJ276" s="4"/>
     </row>
-    <row r="277" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A277" s="3">
         <v>118659</v>
       </c>
@@ -32074,7 +32094,7 @@
       </c>
       <c r="AJ277" s="4"/>
     </row>
-    <row r="278" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A278" s="3">
         <v>117403</v>
       </c>
@@ -32356,7 +32376,7 @@
       </c>
       <c r="AJ280" s="4"/>
     </row>
-    <row r="281" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A281" s="3">
         <v>119932</v>
       </c>
@@ -32450,7 +32470,7 @@
       </c>
       <c r="AJ281" s="4"/>
     </row>
-    <row r="282" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A282" s="3">
         <v>121305</v>
       </c>
@@ -32638,7 +32658,7 @@
       </c>
       <c r="AJ283" s="4"/>
     </row>
-    <row r="284" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A284" s="3">
         <v>108601</v>
       </c>
@@ -32732,7 +32752,7 @@
       </c>
       <c r="AJ284" s="4"/>
     </row>
-    <row r="285" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A285" s="3">
         <v>120639</v>
       </c>
@@ -32824,7 +32844,7 @@
       </c>
       <c r="AJ285" s="4"/>
     </row>
-    <row r="286" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A286" s="3">
         <v>116998</v>
       </c>
@@ -32918,7 +32938,7 @@
       </c>
       <c r="AJ286" s="4"/>
     </row>
-    <row r="287" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A287" s="3">
         <v>115858</v>
       </c>
@@ -33014,7 +33034,7 @@
       </c>
       <c r="AJ287" s="4"/>
     </row>
-    <row r="288" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A288" s="3">
         <v>121520</v>
       </c>
@@ -33112,7 +33132,7 @@
       </c>
       <c r="AJ288" s="4"/>
     </row>
-    <row r="289" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A289" s="3">
         <v>116987</v>
       </c>
@@ -33206,7 +33226,7 @@
       </c>
       <c r="AJ289" s="4"/>
     </row>
-    <row r="290" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A290" s="3">
         <v>121468</v>
       </c>
@@ -33298,7 +33318,7 @@
       </c>
       <c r="AJ290" s="4"/>
     </row>
-    <row r="291" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A291" s="3">
         <v>123190</v>
       </c>
@@ -33488,7 +33508,7 @@
       </c>
       <c r="AJ292" s="4"/>
     </row>
-    <row r="293" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A293" s="3">
         <v>122043</v>
       </c>
@@ -33580,7 +33600,7 @@
       </c>
       <c r="AJ293" s="4"/>
     </row>
-    <row r="294" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A294" s="3">
         <v>121325</v>
       </c>
@@ -33676,7 +33696,7 @@
       </c>
       <c r="AJ294" s="4"/>
     </row>
-    <row r="295" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A295" s="3">
         <v>116467</v>
       </c>
@@ -33864,7 +33884,7 @@
       </c>
       <c r="AJ296" s="4"/>
     </row>
-    <row r="297" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A297" s="3">
         <v>107982</v>
       </c>
@@ -33958,7 +33978,7 @@
       </c>
       <c r="AJ297" s="4"/>
     </row>
-    <row r="298" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A298" s="3">
         <v>108098</v>
       </c>
@@ -34052,7 +34072,7 @@
       </c>
       <c r="AJ298" s="4"/>
     </row>
-    <row r="299" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A299" s="3">
         <v>117041</v>
       </c>
@@ -34144,7 +34164,7 @@
       </c>
       <c r="AJ299" s="4"/>
     </row>
-    <row r="300" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A300" s="3">
         <v>114020</v>
       </c>
@@ -34238,7 +34258,7 @@
       </c>
       <c r="AJ300" s="4"/>
     </row>
-    <row r="301" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A301" s="3">
         <v>108028</v>
       </c>
@@ -34334,7 +34354,7 @@
       </c>
       <c r="AJ301" s="4"/>
     </row>
-    <row r="302" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A302" s="3">
         <v>114019</v>
       </c>
@@ -34428,7 +34448,7 @@
       </c>
       <c r="AJ302" s="4"/>
     </row>
-    <row r="303" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A303" s="3">
         <v>108542</v>
       </c>
@@ -34524,7 +34544,7 @@
       </c>
       <c r="AJ303" s="4"/>
     </row>
-    <row r="304" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A304" s="3">
         <v>117347</v>
       </c>
@@ -34620,7 +34640,7 @@
       </c>
       <c r="AJ304" s="4"/>
     </row>
-    <row r="305" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A305" s="3">
         <v>114596</v>
       </c>
@@ -34716,7 +34736,7 @@
       </c>
       <c r="AJ305" s="4"/>
     </row>
-    <row r="306" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A306" s="3">
         <v>121698</v>
       </c>
@@ -34812,7 +34832,7 @@
       </c>
       <c r="AJ306" s="4"/>
     </row>
-    <row r="307" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A307" s="3">
         <v>108072</v>
       </c>
@@ -34908,7 +34928,7 @@
       </c>
       <c r="AJ307" s="4"/>
     </row>
-    <row r="308" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A308" s="3">
         <v>123111</v>
       </c>
@@ -35000,7 +35020,7 @@
       </c>
       <c r="AJ308" s="4"/>
     </row>
-    <row r="309" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A309" s="3">
         <v>120559</v>
       </c>
@@ -35192,7 +35212,7 @@
       </c>
       <c r="AJ310" s="4"/>
     </row>
-    <row r="311" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A311" s="3">
         <v>112113</v>
       </c>
@@ -35286,7 +35306,7 @@
       </c>
       <c r="AJ311" s="4"/>
     </row>
-    <row r="312" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A312" s="3">
         <v>115034</v>
       </c>
@@ -35382,7 +35402,7 @@
       </c>
       <c r="AJ312" s="4"/>
     </row>
-    <row r="313" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A313" s="3">
         <v>114727</v>
       </c>
@@ -35476,7 +35496,7 @@
       </c>
       <c r="AJ313" s="4"/>
     </row>
-    <row r="314" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A314" s="3">
         <v>106674</v>
       </c>
@@ -35570,7 +35590,7 @@
       </c>
       <c r="AJ314" s="4"/>
     </row>
-    <row r="315" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A315" s="3">
         <v>111207</v>
       </c>
@@ -35666,7 +35686,7 @@
       </c>
       <c r="AJ315" s="4"/>
     </row>
-    <row r="316" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A316" s="3">
         <v>114791</v>
       </c>
@@ -35760,7 +35780,7 @@
       </c>
       <c r="AJ316" s="4"/>
     </row>
-    <row r="317" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A317" s="3">
         <v>107375</v>
       </c>
@@ -35856,7 +35876,7 @@
       </c>
       <c r="AJ317" s="4"/>
     </row>
-    <row r="318" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A318" s="3">
         <v>109086</v>
       </c>
@@ -35952,7 +35972,7 @@
       </c>
       <c r="AJ318" s="4"/>
     </row>
-    <row r="319" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A319" s="3">
         <v>114730</v>
       </c>
@@ -36046,7 +36066,7 @@
       </c>
       <c r="AJ319" s="4"/>
     </row>
-    <row r="320" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A320" s="3">
         <v>109604</v>
       </c>
@@ -36140,7 +36160,7 @@
       </c>
       <c r="AJ320" s="4"/>
     </row>
-    <row r="321" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A321" s="3">
         <v>113929</v>
       </c>
@@ -36330,7 +36350,7 @@
       </c>
       <c r="AJ322" s="4"/>
     </row>
-    <row r="323" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A323" s="3">
         <v>114005</v>
       </c>
@@ -36424,7 +36444,7 @@
       </c>
       <c r="AJ323" s="4"/>
     </row>
-    <row r="324" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A324" s="3">
         <v>111252</v>
       </c>
@@ -36518,7 +36538,7 @@
       </c>
       <c r="AJ324" s="4"/>
     </row>
-    <row r="325" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A325" s="3">
         <v>107928</v>
       </c>
@@ -36614,7 +36634,7 @@
       </c>
       <c r="AJ325" s="4"/>
     </row>
-    <row r="326" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A326" s="3">
         <v>111805</v>
       </c>
@@ -36708,7 +36728,7 @@
       </c>
       <c r="AJ326" s="4"/>
     </row>
-    <row r="327" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A327" s="3">
         <v>115143</v>
       </c>
@@ -36804,7 +36824,7 @@
       </c>
       <c r="AJ327" s="4"/>
     </row>
-    <row r="328" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A328" s="3">
         <v>109349</v>
       </c>
@@ -36902,7 +36922,7 @@
       </c>
       <c r="AJ328" s="4"/>
     </row>
-    <row r="329" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A329" s="3">
         <v>112503</v>
       </c>
@@ -37090,7 +37110,7 @@
       </c>
       <c r="AJ330" s="4"/>
     </row>
-    <row r="331" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A331" s="3">
         <v>112796</v>
       </c>
@@ -37278,7 +37298,7 @@
       </c>
       <c r="AJ332" s="4"/>
     </row>
-    <row r="333" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A333" s="3">
         <v>113446</v>
       </c>
@@ -37942,7 +37962,7 @@
       </c>
       <c r="AJ339" s="4"/>
     </row>
-    <row r="340" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A340" s="3">
         <v>107703</v>
       </c>
@@ -38038,7 +38058,7 @@
       </c>
       <c r="AJ340" s="4"/>
     </row>
-    <row r="341" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A341" s="3">
         <v>120997</v>
       </c>
@@ -38132,7 +38152,7 @@
       </c>
       <c r="AJ341" s="4"/>
     </row>
-    <row r="342" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A342" s="3">
         <v>121143</v>
       </c>
@@ -38694,7 +38714,7 @@
       </c>
       <c r="AJ347" s="4"/>
     </row>
-    <row r="348" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A348" s="3">
         <v>121135</v>
       </c>
@@ -38788,7 +38808,7 @@
       </c>
       <c r="AJ348" s="4"/>
     </row>
-    <row r="349" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A349" s="3">
         <v>122038</v>
       </c>
@@ -38884,7 +38904,7 @@
       </c>
       <c r="AJ349" s="4"/>
     </row>
-    <row r="350" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A350" s="3">
         <v>123143</v>
       </c>
@@ -38976,7 +38996,7 @@
       </c>
       <c r="AJ350" s="4"/>
     </row>
-    <row r="351" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A351" s="3">
         <v>121408</v>
       </c>
@@ -39070,7 +39090,7 @@
       </c>
       <c r="AJ351" s="4"/>
     </row>
-    <row r="352" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A352" s="3">
         <v>113591</v>
       </c>
@@ -39164,7 +39184,7 @@
       </c>
       <c r="AJ352" s="4"/>
     </row>
-    <row r="353" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A353" s="3">
         <v>120365</v>
       </c>
@@ -39352,7 +39372,7 @@
       </c>
       <c r="AJ354" s="4"/>
     </row>
-    <row r="355" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A355" s="3">
         <v>120796</v>
       </c>
@@ -39446,7 +39466,7 @@
       </c>
       <c r="AJ355" s="4"/>
     </row>
-    <row r="356" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A356" s="3">
         <v>121202</v>
       </c>
@@ -39542,7 +39562,7 @@
       </c>
       <c r="AJ356" s="4"/>
     </row>
-    <row r="357" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A357" s="3">
         <v>121989</v>
       </c>
@@ -39638,7 +39658,7 @@
       </c>
       <c r="AJ357" s="4"/>
     </row>
-    <row r="358" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A358" s="3">
         <v>122051</v>
       </c>
@@ -39826,7 +39846,7 @@
       </c>
       <c r="AJ359" s="4"/>
     </row>
-    <row r="360" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A360" s="3">
         <v>122018</v>
       </c>
@@ -39920,7 +39940,7 @@
       </c>
       <c r="AJ360" s="4"/>
     </row>
-    <row r="361" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A361" s="3">
         <v>122102</v>
       </c>
@@ -40014,7 +40034,7 @@
       </c>
       <c r="AJ361" s="4"/>
     </row>
-    <row r="362" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A362" s="3">
         <v>121976</v>
       </c>
@@ -40108,7 +40128,7 @@
       </c>
       <c r="AJ362" s="4"/>
     </row>
-    <row r="363" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A363" s="3">
         <v>121288</v>
       </c>
@@ -40204,7 +40224,7 @@
       </c>
       <c r="AJ363" s="4"/>
     </row>
-    <row r="364" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A364" s="3">
         <v>120005</v>
       </c>
@@ -40300,7 +40320,7 @@
       </c>
       <c r="AJ364" s="4"/>
     </row>
-    <row r="365" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A365" s="3">
         <v>120004</v>
       </c>
@@ -40394,7 +40414,7 @@
       </c>
       <c r="AJ365" s="4"/>
     </row>
-    <row r="366" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A366" s="3">
         <v>116827</v>
       </c>
@@ -40490,7 +40510,7 @@
       </c>
       <c r="AJ366" s="4"/>
     </row>
-    <row r="367" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A367" s="3">
         <v>113155</v>
       </c>
@@ -40584,7 +40604,7 @@
       </c>
       <c r="AJ367" s="4"/>
     </row>
-    <row r="368" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A368" s="3">
         <v>113970</v>
       </c>
@@ -40680,7 +40700,7 @@
       </c>
       <c r="AJ368" s="4"/>
     </row>
-    <row r="369" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A369" s="3">
         <v>116634</v>
       </c>
@@ -40776,7 +40796,7 @@
       </c>
       <c r="AJ369" s="4"/>
     </row>
-    <row r="370" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A370" s="3">
         <v>116622</v>
       </c>
@@ -40966,7 +40986,7 @@
       </c>
       <c r="AJ371" s="4"/>
     </row>
-    <row r="372" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A372" s="3">
         <v>113121</v>
       </c>
@@ -41060,7 +41080,7 @@
       </c>
       <c r="AJ372" s="4"/>
     </row>
-    <row r="373" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A373" s="3">
         <v>116662</v>
       </c>
@@ -41254,7 +41274,7 @@
       </c>
       <c r="AJ374" s="4"/>
     </row>
-    <row r="375" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A375" s="3">
         <v>112661</v>
       </c>
@@ -41348,7 +41368,7 @@
       </c>
       <c r="AJ375" s="4"/>
     </row>
-    <row r="376" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A376" s="3">
         <v>111339</v>
       </c>
@@ -41444,7 +41464,7 @@
       </c>
       <c r="AJ376" s="4"/>
     </row>
-    <row r="377" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A377" s="3">
         <v>113878</v>
       </c>
@@ -41540,7 +41560,7 @@
       </c>
       <c r="AJ377" s="4"/>
     </row>
-    <row r="378" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A378" s="3">
         <v>107151</v>
       </c>
@@ -41636,7 +41656,7 @@
       </c>
       <c r="AJ378" s="4"/>
     </row>
-    <row r="379" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A379" s="3">
         <v>113196</v>
       </c>
@@ -41730,7 +41750,7 @@
       </c>
       <c r="AJ379" s="4"/>
     </row>
-    <row r="380" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A380" s="3">
         <v>122024</v>
       </c>
@@ -41824,7 +41844,7 @@
       </c>
       <c r="AJ380" s="4"/>
     </row>
-    <row r="381" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A381" s="3">
         <v>115992</v>
       </c>
@@ -41918,7 +41938,7 @@
       </c>
       <c r="AJ381" s="4"/>
     </row>
-    <row r="382" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A382" s="3">
         <v>122105</v>
       </c>
@@ -42010,7 +42030,7 @@
       </c>
       <c r="AJ382" s="4"/>
     </row>
-    <row r="383" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A383" s="3">
         <v>112134</v>
       </c>
@@ -42388,7 +42408,7 @@
       </c>
       <c r="AJ386" s="4"/>
     </row>
-    <row r="387" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="387" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A387" s="3">
         <v>117636</v>
       </c>
@@ -42576,7 +42596,7 @@
       </c>
       <c r="AJ388" s="4"/>
     </row>
-    <row r="389" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="389" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A389" s="3">
         <v>115459</v>
       </c>
@@ -42668,7 +42688,7 @@
       </c>
       <c r="AJ389" s="4"/>
     </row>
-    <row r="390" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="390" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A390" s="3">
         <v>118754</v>
       </c>
@@ -42764,7 +42784,7 @@
       </c>
       <c r="AJ390" s="4"/>
     </row>
-    <row r="391" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="391" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A391" s="3">
         <v>109174</v>
       </c>
@@ -42860,7 +42880,7 @@
       </c>
       <c r="AJ391" s="4"/>
     </row>
-    <row r="392" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="392" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A392" s="3">
         <v>116282</v>
       </c>
@@ -43048,7 +43068,7 @@
       </c>
       <c r="AJ393" s="4"/>
     </row>
-    <row r="394" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="394" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A394" s="3">
         <v>110451</v>
       </c>
@@ -43142,7 +43162,7 @@
       </c>
       <c r="AJ394" s="4"/>
     </row>
-    <row r="395" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="395" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A395" s="3">
         <v>117974</v>
       </c>
@@ -43236,7 +43256,7 @@
       </c>
       <c r="AJ395" s="4"/>
     </row>
-    <row r="396" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="396" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A396" s="3">
         <v>108851</v>
       </c>
@@ -43332,7 +43352,7 @@
       </c>
       <c r="AJ396" s="4"/>
     </row>
-    <row r="397" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="397" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A397" s="3">
         <v>115940</v>
       </c>
@@ -43426,7 +43446,7 @@
       </c>
       <c r="AJ397" s="4"/>
     </row>
-    <row r="398" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="398" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A398" s="3">
         <v>112683</v>
       </c>
@@ -43522,7 +43542,7 @@
       </c>
       <c r="AJ398" s="4"/>
     </row>
-    <row r="399" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="399" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A399" s="3">
         <v>115936</v>
       </c>
@@ -43802,7 +43822,7 @@
       </c>
       <c r="AJ401" s="4"/>
     </row>
-    <row r="402" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="402" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A402" s="3">
         <v>108788</v>
       </c>
@@ -43992,7 +44012,7 @@
       </c>
       <c r="AJ403" s="4"/>
     </row>
-    <row r="404" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="404" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A404" s="3">
         <v>118036</v>
       </c>
@@ -44086,7 +44106,7 @@
       </c>
       <c r="AJ404" s="4"/>
     </row>
-    <row r="405" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="405" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A405" s="3">
         <v>113858</v>
       </c>
@@ -44178,7 +44198,7 @@
       </c>
       <c r="AJ405" s="4"/>
     </row>
-    <row r="406" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="406" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A406" s="3">
         <v>116611</v>
       </c>
@@ -44460,7 +44480,7 @@
       </c>
       <c r="AJ408" s="4"/>
     </row>
-    <row r="409" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="409" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A409" s="3">
         <v>116692</v>
       </c>
@@ -44554,7 +44574,7 @@
       </c>
       <c r="AJ409" s="4"/>
     </row>
-    <row r="410" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="410" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A410" s="3">
         <v>117934</v>
       </c>
@@ -44648,7 +44668,7 @@
       </c>
       <c r="AJ410" s="4"/>
     </row>
-    <row r="411" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="411" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A411" s="3">
         <v>116629</v>
       </c>
@@ -44744,7 +44764,7 @@
       </c>
       <c r="AJ411" s="4"/>
     </row>
-    <row r="412" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="412" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A412" s="3">
         <v>115574</v>
       </c>
@@ -44838,7 +44858,7 @@
       </c>
       <c r="AJ412" s="4"/>
     </row>
-    <row r="413" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="413" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A413" s="3">
         <v>118987</v>
       </c>
@@ -44932,7 +44952,7 @@
       </c>
       <c r="AJ413" s="4"/>
     </row>
-    <row r="414" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="414" spans="1:36" hidden="1" x14ac:dyDescent="0.25">
       <c r="A414" s="3">
         <v>119923</v>
       </c>
@@ -45027,6 +45047,13 @@
       <c r="AJ414" s="4"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:AJ414" xr:uid="{86915FE4-2993-48FB-9CAA-1D0CCEED47A1}">
+    <filterColumn colId="11">
+      <filters>
+        <filter val="MONITOR DE SIGNOS VITALES"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>